<commit_message>
updated Api key and added logger
</commit_message>
<xml_diff>
--- a/CapstoneScenario3PostmanApiAutomation/src/test/resources/credentials.xlsx
+++ b/CapstoneScenario3PostmanApiAutomation/src/test/resources/credentials.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sahasra Reddy\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Capstone\CapstoneScenario3PostmanApiAutomation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2416B94-9DE6-45AE-9D2F-4B9DDBD2DBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84664550-FBAE-453C-8393-F9D5F05B6923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1702676D-D848-4DB3-A129-C39DD3B3E8C4}"/>
   </bookViews>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,24 +34,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test1@example.com </t>
-  </si>
-  <si>
-    <t xml:space="preserve">test2@example.com </t>
-  </si>
-  <si>
-    <t>password1</t>
-  </si>
-  <si>
-    <t>password2</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>eve.holt@reqres.in</t>
+  </si>
+  <si>
+    <t>pistol</t>
+  </si>
+  <si>
+    <t>missing.password@reqres.in</t>
+  </si>
+  <si>
+    <t>invalid.email@reqres.in</t>
+  </si>
+  <si>
+    <t>wrongpass</t>
   </si>
 </sst>
 </file>
@@ -419,8 +420,8 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="1" max="1" width="31.453125" customWidth="1"/>
+    <col min="2" max="2" width="14.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -436,24 +437,23 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A3" r:id="rId1" xr:uid="{865D5173-77FB-4E5B-8396-67476DCE2143}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>